<commit_message>
removed two carbon source cultivation
</commit_message>
<xml_diff>
--- a/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
+++ b/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
@@ -8,7 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Aerobic" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Anaerobic" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
   <si>
     <t xml:space="preserve">Growth</t>
   </si>
@@ -88,6 +89,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -109,23 +111,27 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF6AAB73"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -272,8 +278,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ11"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -306,8 +312,9 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AMJ1" s="0"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="n">
         <v>0.59</v>
       </c>
@@ -339,7 +346,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>0.48</v>
       </c>
@@ -371,7 +378,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
         <v>0.61</v>
       </c>
@@ -403,7 +410,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>0.443</v>
       </c>
@@ -435,15 +442,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
-        <v>0.52</v>
+        <v>0.43</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>-3.36</v>
+        <v>-5.4</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>-3.12</v>
+        <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>0</v>
@@ -467,15 +474,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
-        <v>0.43</v>
+        <v>0.46</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>-5.4</v>
+        <v>0</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0</v>
+        <v>-5.88</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>0</v>
@@ -487,7 +494,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>10</v>
@@ -499,15 +506,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
-        <v>0.46</v>
+        <v>0.2</v>
       </c>
       <c r="B8" s="4" t="n">
-        <v>0</v>
+        <v>-2.33</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>5.88</v>
+        <v>0</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>0</v>
@@ -519,24 +526,24 @@
         <v>0</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>10</v>
+        <v>5.36</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>10</v>
+        <v>5.64</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>14</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="B9" s="4" t="n">
-        <v>2.33</v>
+        <v>-3.44</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>0</v>
@@ -551,10 +558,10 @@
         <v>0</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>5.36</v>
+        <v>7.16</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>5.64</v>
+        <v>7.3</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>14</v>
@@ -563,12 +570,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="B10" s="4" t="n">
-        <v>3.44</v>
+        <v>-4.27</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>0</v>
@@ -583,10 +590,10 @@
         <v>0</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>7.16</v>
+        <v>8.15</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>7.3</v>
+        <v>7.94</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>14</v>
@@ -595,12 +602,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="B11" s="4" t="n">
-        <v>4.27</v>
+        <v>0</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>0</v>
@@ -612,50 +619,18 @@
         <v>0</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0</v>
+        <v>-24</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>8.15</v>
+        <v>10</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>7.94</v>
+        <v>10</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>14</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="J12" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -668,4 +643,22 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
improved parsing of validation data for cglutanicum
</commit_message>
<xml_diff>
--- a/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
+++ b/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
@@ -32,7 +32,7 @@
     <t xml:space="preserve">EX_glcn_e</t>
   </si>
   <si>
-    <t xml:space="preserve">EX_sucs_e</t>
+    <t xml:space="preserve">EX_succ_e</t>
   </si>
   <si>
     <t xml:space="preserve">EX_fru_e</t>
@@ -311,14 +311,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ19"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.56"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="11.56"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="29.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30.7"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.56"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.57"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -982,7 +982,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
removed default co2 and o2 exchange values when not reported
</commit_message>
<xml_diff>
--- a/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
+++ b/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
@@ -311,7 +311,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ19"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.11"/>
@@ -376,12 +376,8 @@
       <c r="F2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>-10</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>10</v>
-      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
       <c r="I2" s="6" t="s">
         <v>11</v>
       </c>
@@ -409,12 +405,8 @@
       <c r="F3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>-10</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>10</v>
-      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
       <c r="I3" s="6" t="s">
         <v>11</v>
       </c>
@@ -442,12 +434,8 @@
       <c r="F4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="5" t="n">
-        <v>-10</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>10</v>
-      </c>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
       <c r="I4" s="6" t="s">
         <v>11</v>
       </c>
@@ -475,12 +463,8 @@
       <c r="F5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="5" t="n">
-        <v>-10</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>10</v>
-      </c>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
       <c r="I5" s="6" t="s">
         <v>13</v>
       </c>
@@ -508,12 +492,8 @@
       <c r="F6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>-10</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>10</v>
-      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
       <c r="I6" s="6" t="s">
         <v>15</v>
       </c>
@@ -541,12 +521,8 @@
       <c r="F7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>10</v>
-      </c>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="6" t="s">
         <v>15</v>
       </c>
@@ -673,12 +649,8 @@
       <c r="F11" s="5" t="n">
         <v>-24</v>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>10</v>
-      </c>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
       <c r="I11" s="6" t="s">
         <v>15</v>
       </c>
@@ -982,7 +954,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
added growth rate to mfa measurements
</commit_message>
<xml_diff>
--- a/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
+++ b/Data/Cglutanicum_phenotypes/cglutanicum_phenotypes.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="45">
   <si>
     <t xml:space="preserve">quantitative physiology measurements for Corynebacterium glutanicum ATC13032 </t>
   </si>
@@ -166,7 +166,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -224,6 +224,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -273,7 +279,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -316,6 +322,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -396,7 +406,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -439,7 +449,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ19"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="16.11"/>
@@ -1081,8 +1091,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:R3"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
@@ -1134,6 +1144,9 @@
         <v>41</v>
       </c>
       <c r="Q1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="R1" s="6" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1186,11 +1199,15 @@
       <c r="P2" s="1" t="n">
         <v>0.449</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="Q2" s="0" t="n">
+        <f aca="false">Q3/A3</f>
+        <v>0.0948608137044968</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>4.67</v>
       </c>
@@ -1254,7 +1271,10 @@
         <f aca="false">P2*A3</f>
         <v>2.09683</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="Q3" s="11" t="n">
+        <v>0.443</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>